<commit_message>
BWI sync — 2026-09-28 09:11 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA337"/>
+  <dimension ref="A1:AA338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -32982,6 +32982,95 @@
       <c r="Z337" s="2" t="inlineStr"/>
       <c r="AA337" s="2" t="inlineStr"/>
     </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>Digimpex Srl</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>Digimpex Srl</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>46195</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>Wilde</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G338" s="2" t="inlineStr">
+        <is>
+          <t>6224 Mariano Moreno</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr">
+        <is>
+          <t>B1875</t>
+        </is>
+      </c>
+      <c r="I338" s="2" t="inlineStr">
+        <is>
+          <t>https://digimpex.com</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr"/>
+      <c r="K338" s="2" t="inlineStr"/>
+      <c r="L338" s="2" t="inlineStr"/>
+      <c r="M338" s="2" t="inlineStr"/>
+      <c r="N338" s="2" t="inlineStr">
+        <is>
+          <t>digimpex@gmail.com</t>
+        </is>
+      </c>
+      <c r="O338" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 4206-1087</t>
+        </is>
+      </c>
+      <c r="P338" s="2" t="inlineStr"/>
+      <c r="Q338" s="2" t="inlineStr"/>
+      <c r="R338" s="2" t="inlineStr"/>
+      <c r="S338" s="2" t="inlineStr"/>
+      <c r="T338" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/digimpexsrl</t>
+        </is>
+      </c>
+      <c r="U338" s="2" t="inlineStr"/>
+      <c r="V338" s="2" t="inlineStr"/>
+      <c r="W338" s="2" t="inlineStr">
+        <is>
+          <t>Marco Di Meo</t>
+        </is>
+      </c>
+      <c r="X338" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="Y338" s="2" t="inlineStr"/>
+      <c r="Z338" s="2" t="inlineStr"/>
+      <c r="AA338" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/marco-di-meo-55144b35/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-10-05 09:18 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Argentina.xlsx
+++ b/BWI/bestwine_output/bestwine_Argentina.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA338"/>
+  <dimension ref="A1:AA342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -33071,6 +33071,422 @@
         </is>
       </c>
     </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>Espaciovino S.r.l.</t>
+        </is>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>Espaciovino</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>CABA</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="G339" s="2" t="inlineStr">
+        <is>
+          <t>Santo Tomé 3852</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr">
+        <is>
+          <t>C1417</t>
+        </is>
+      </c>
+      <c r="I339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.espaciovino.com.ar</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr"/>
+      <c r="K339" s="2" t="inlineStr"/>
+      <c r="L339" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M339" s="2" t="inlineStr"/>
+      <c r="N339" s="2" t="inlineStr">
+        <is>
+          <t>info@espaciovino.com.ar</t>
+        </is>
+      </c>
+      <c r="O339" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 5352-8466</t>
+        </is>
+      </c>
+      <c r="P339" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="Q339" s="2" t="inlineStr">
+        <is>
+          <t>30-71564031-3</t>
+        </is>
+      </c>
+      <c r="R339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/espaciovino-com/</t>
+        </is>
+      </c>
+      <c r="S339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/espaciovino/</t>
+        </is>
+      </c>
+      <c r="T339" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/espaciovino</t>
+        </is>
+      </c>
+      <c r="U339" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/espaciovino</t>
+        </is>
+      </c>
+      <c r="V339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@espaciovinoAr/</t>
+        </is>
+      </c>
+      <c r="W339" s="2" t="inlineStr">
+        <is>
+          <t>Martin Fernandez</t>
+        </is>
+      </c>
+      <c r="X339" s="2" t="inlineStr">
+        <is>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="Y339" s="2" t="inlineStr"/>
+      <c r="Z339" s="2" t="inlineStr"/>
+      <c r="AA339" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/martinf/</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>Espaciovino S.r.l.</t>
+        </is>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>Espaciovino</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>CABA</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="G340" s="2" t="inlineStr">
+        <is>
+          <t>Santo Tomé 3852</t>
+        </is>
+      </c>
+      <c r="H340" s="2" t="inlineStr">
+        <is>
+          <t>C1417</t>
+        </is>
+      </c>
+      <c r="I340" s="2" t="inlineStr">
+        <is>
+          <t>https://www.espaciovino.com.ar</t>
+        </is>
+      </c>
+      <c r="J340" s="2" t="inlineStr"/>
+      <c r="K340" s="2" t="inlineStr"/>
+      <c r="L340" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M340" s="2" t="inlineStr"/>
+      <c r="N340" s="2" t="inlineStr">
+        <is>
+          <t>info@espaciovino.com.ar</t>
+        </is>
+      </c>
+      <c r="O340" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 5352-8466</t>
+        </is>
+      </c>
+      <c r="P340" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="Q340" s="2" t="inlineStr">
+        <is>
+          <t>30-71564031-3</t>
+        </is>
+      </c>
+      <c r="R340" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/espaciovino-com/</t>
+        </is>
+      </c>
+      <c r="S340" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/espaciovino/</t>
+        </is>
+      </c>
+      <c r="T340" s="2" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/espaciovino</t>
+        </is>
+      </c>
+      <c r="U340" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/espaciovino</t>
+        </is>
+      </c>
+      <c r="V340" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@espaciovinoAr/</t>
+        </is>
+      </c>
+      <c r="W340" s="2" t="inlineStr">
+        <is>
+          <t>Diego Fernández</t>
+        </is>
+      </c>
+      <c r="X340" s="2" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="Y340" s="2" t="inlineStr"/>
+      <c r="Z340" s="2" t="inlineStr"/>
+      <c r="AA340" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/diego-fern%C3%A1ndez-058b3b95/</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>Little Italia Market</t>
+        </is>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>Little Italia Market</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>122576</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>Autonomous City of Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G341" s="2" t="inlineStr">
+        <is>
+          <t>2701 Doctor Rómulo Naón</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="inlineStr">
+        <is>
+          <t>C1430</t>
+        </is>
+      </c>
+      <c r="I341" s="2" t="inlineStr">
+        <is>
+          <t>https://littleitaliamarket.com.ar</t>
+        </is>
+      </c>
+      <c r="J341" s="2" t="inlineStr"/>
+      <c r="K341" s="2" t="inlineStr"/>
+      <c r="L341" s="2" t="inlineStr"/>
+      <c r="M341" s="2" t="inlineStr"/>
+      <c r="N341" s="2" t="inlineStr">
+        <is>
+          <t>italianmarket20@gmail.com</t>
+        </is>
+      </c>
+      <c r="O341" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 3132-8558</t>
+        </is>
+      </c>
+      <c r="P341" s="2" t="inlineStr"/>
+      <c r="Q341" s="2" t="inlineStr"/>
+      <c r="R341" s="2" t="inlineStr"/>
+      <c r="S341" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Littleitaliamarket/</t>
+        </is>
+      </c>
+      <c r="T341" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/littleitaliamarket/</t>
+        </is>
+      </c>
+      <c r="U341" s="2" t="inlineStr"/>
+      <c r="V341" s="2" t="inlineStr"/>
+      <c r="W341" s="2" t="inlineStr">
+        <is>
+          <t>Luciano Arias</t>
+        </is>
+      </c>
+      <c r="X341" s="2" t="inlineStr">
+        <is>
+          <t>Sales Specialist</t>
+        </is>
+      </c>
+      <c r="Y341" s="2" t="inlineStr"/>
+      <c r="Z341" s="2" t="inlineStr"/>
+      <c r="AA341" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/luciano-arias-a80066274/</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>Digimpex Srl</t>
+        </is>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>Digimpex Srl</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>46195</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>Wilde</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="G342" s="2" t="inlineStr">
+        <is>
+          <t>6224 Mariano Moreno</t>
+        </is>
+      </c>
+      <c r="H342" s="2" t="inlineStr">
+        <is>
+          <t>B1875</t>
+        </is>
+      </c>
+      <c r="I342" s="2" t="inlineStr">
+        <is>
+          <t>https://digimpex.com</t>
+        </is>
+      </c>
+      <c r="J342" s="2" t="inlineStr"/>
+      <c r="K342" s="2" t="inlineStr"/>
+      <c r="L342" s="2" t="inlineStr"/>
+      <c r="M342" s="2" t="inlineStr"/>
+      <c r="N342" s="2" t="inlineStr">
+        <is>
+          <t>digimpex@gmail.com</t>
+        </is>
+      </c>
+      <c r="O342" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 4206-1087</t>
+        </is>
+      </c>
+      <c r="P342" s="2" t="inlineStr"/>
+      <c r="Q342" s="2" t="inlineStr"/>
+      <c r="R342" s="2" t="inlineStr"/>
+      <c r="S342" s="2" t="inlineStr"/>
+      <c r="T342" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/digimpexsrl</t>
+        </is>
+      </c>
+      <c r="U342" s="2" t="inlineStr"/>
+      <c r="V342" s="2" t="inlineStr"/>
+      <c r="W342" s="2" t="inlineStr">
+        <is>
+          <t>Marco Di Meo</t>
+        </is>
+      </c>
+      <c r="X342" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="Y342" s="2" t="inlineStr"/>
+      <c r="Z342" s="2" t="inlineStr"/>
+      <c r="AA342" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/marco-di-meo-55144b35/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>